<commit_message>
Add request status (New / In process / Done / Cancelled), v1.2.0
- Status picker in the form, an inline status drop-down in every row,
  a status filter and an "In process" counter
- Excel: Status column with one colour per value and a drop-down list
- Changing a status also rewrites the Status cell in every exported
  Excel file holding that row; the file search editor offers the same list
- Linux service accepts the new field; README documents updating

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ACP4U-Parts-Form.xlsx
+++ b/ACP4U-Parts-Form.xlsx
@@ -9,7 +9,7 @@
     <sheet name="Parts Requests" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Parts Requests'!$A$3:$O$33</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Parts Requests'!$A$3:$P$33</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Parts Requests'!$1:$3</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
   <si>
     <r>
       <rPr>
@@ -72,6 +72,9 @@
   </si>
   <si>
     <t xml:space="preserve">Required Part</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Status</t>
   </si>
   <si>
     <t xml:space="preserve">Photo 1</t>
@@ -315,7 +318,52 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="4">
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF1F4E79"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFDDEBF7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF6B7280"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFE5E7EB"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
 </styleSheet>
 </file>
@@ -326,7 +374,7 @@
     <tabColor rgb="FFF57C1F"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O33"/>
+  <dimension ref="A1:P33"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="7" customWidth="1"/>
@@ -339,11 +387,12 @@
     <col min="8" max="8" width="9" customWidth="1"/>
     <col min="9" max="9" width="24" customWidth="1"/>
     <col min="10" max="10" width="32" customWidth="1"/>
-    <col min="11" max="11" width="18" customWidth="1"/>
+    <col min="11" max="11" width="14" customWidth="1"/>
     <col min="12" max="12" width="18" customWidth="1"/>
     <col min="13" max="13" width="18" customWidth="1"/>
     <col min="14" max="14" width="18" customWidth="1"/>
     <col min="15" max="15" width="18" customWidth="1"/>
+    <col min="16" max="16" width="18" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="40" customHeight="1">
@@ -364,6 +413,7 @@
       <c r="M1" s="1"/>
       <c r="N1" s="1"/>
       <c r="O1" s="1"/>
+      <c r="P1" s="1"/>
     </row>
     <row r="2" ht="24" customHeight="1">
       <c r="A2" s="2" t="s">
@@ -383,6 +433,7 @@
       <c r="M2" s="2"/>
       <c r="N2" s="2"/>
       <c r="O2" s="2"/>
+      <c r="P2" s="2"/>
     </row>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="3" t="s">
@@ -415,7 +466,7 @@
       <c r="J3" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="K3" s="4" t="s">
+      <c r="K3" s="3" t="s">
         <v>12</v>
       </c>
       <c r="L3" s="4" t="s">
@@ -429,6 +480,9 @@
       </c>
       <c r="O3" s="4" t="s">
         <v>16</v>
+      </c>
+      <c r="P3" s="4" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="4" ht="84" customHeight="1">
@@ -444,11 +498,12 @@
       <c r="H4" s="7"/>
       <c r="I4" s="9"/>
       <c r="J4" s="11"/>
-      <c r="K4" s="13"/>
+      <c r="K4" s="7"/>
       <c r="L4" s="13"/>
       <c r="M4" s="13"/>
       <c r="N4" s="13"/>
       <c r="O4" s="13"/>
+      <c r="P4" s="13"/>
     </row>
     <row r="5" ht="84" customHeight="1">
       <c r="A5" s="6">
@@ -463,11 +518,12 @@
       <c r="H5" s="8"/>
       <c r="I5" s="10"/>
       <c r="J5" s="12"/>
-      <c r="K5" s="14"/>
+      <c r="K5" s="8"/>
       <c r="L5" s="14"/>
       <c r="M5" s="14"/>
       <c r="N5" s="14"/>
       <c r="O5" s="14"/>
+      <c r="P5" s="14"/>
     </row>
     <row r="6" ht="84" customHeight="1">
       <c r="A6" s="5">
@@ -482,11 +538,12 @@
       <c r="H6" s="7"/>
       <c r="I6" s="9"/>
       <c r="J6" s="11"/>
-      <c r="K6" s="13"/>
+      <c r="K6" s="7"/>
       <c r="L6" s="13"/>
       <c r="M6" s="13"/>
       <c r="N6" s="13"/>
       <c r="O6" s="13"/>
+      <c r="P6" s="13"/>
     </row>
     <row r="7" ht="84" customHeight="1">
       <c r="A7" s="6">
@@ -501,11 +558,12 @@
       <c r="H7" s="8"/>
       <c r="I7" s="10"/>
       <c r="J7" s="12"/>
-      <c r="K7" s="14"/>
+      <c r="K7" s="8"/>
       <c r="L7" s="14"/>
       <c r="M7" s="14"/>
       <c r="N7" s="14"/>
       <c r="O7" s="14"/>
+      <c r="P7" s="14"/>
     </row>
     <row r="8" ht="84" customHeight="1">
       <c r="A8" s="5">
@@ -520,11 +578,12 @@
       <c r="H8" s="7"/>
       <c r="I8" s="9"/>
       <c r="J8" s="11"/>
-      <c r="K8" s="13"/>
+      <c r="K8" s="7"/>
       <c r="L8" s="13"/>
       <c r="M8" s="13"/>
       <c r="N8" s="13"/>
       <c r="O8" s="13"/>
+      <c r="P8" s="13"/>
     </row>
     <row r="9" ht="84" customHeight="1">
       <c r="A9" s="6">
@@ -539,11 +598,12 @@
       <c r="H9" s="8"/>
       <c r="I9" s="10"/>
       <c r="J9" s="12"/>
-      <c r="K9" s="14"/>
+      <c r="K9" s="8"/>
       <c r="L9" s="14"/>
       <c r="M9" s="14"/>
       <c r="N9" s="14"/>
       <c r="O9" s="14"/>
+      <c r="P9" s="14"/>
     </row>
     <row r="10" ht="84" customHeight="1">
       <c r="A10" s="5">
@@ -558,11 +618,12 @@
       <c r="H10" s="7"/>
       <c r="I10" s="9"/>
       <c r="J10" s="11"/>
-      <c r="K10" s="13"/>
+      <c r="K10" s="7"/>
       <c r="L10" s="13"/>
       <c r="M10" s="13"/>
       <c r="N10" s="13"/>
       <c r="O10" s="13"/>
+      <c r="P10" s="13"/>
     </row>
     <row r="11" ht="84" customHeight="1">
       <c r="A11" s="6">
@@ -577,11 +638,12 @@
       <c r="H11" s="8"/>
       <c r="I11" s="10"/>
       <c r="J11" s="12"/>
-      <c r="K11" s="14"/>
+      <c r="K11" s="8"/>
       <c r="L11" s="14"/>
       <c r="M11" s="14"/>
       <c r="N11" s="14"/>
       <c r="O11" s="14"/>
+      <c r="P11" s="14"/>
     </row>
     <row r="12" ht="84" customHeight="1">
       <c r="A12" s="5">
@@ -596,11 +658,12 @@
       <c r="H12" s="7"/>
       <c r="I12" s="9"/>
       <c r="J12" s="11"/>
-      <c r="K12" s="13"/>
+      <c r="K12" s="7"/>
       <c r="L12" s="13"/>
       <c r="M12" s="13"/>
       <c r="N12" s="13"/>
       <c r="O12" s="13"/>
+      <c r="P12" s="13"/>
     </row>
     <row r="13" ht="84" customHeight="1">
       <c r="A13" s="6">
@@ -615,11 +678,12 @@
       <c r="H13" s="8"/>
       <c r="I13" s="10"/>
       <c r="J13" s="12"/>
-      <c r="K13" s="14"/>
+      <c r="K13" s="8"/>
       <c r="L13" s="14"/>
       <c r="M13" s="14"/>
       <c r="N13" s="14"/>
       <c r="O13" s="14"/>
+      <c r="P13" s="14"/>
     </row>
     <row r="14" ht="84" customHeight="1">
       <c r="A14" s="5">
@@ -634,11 +698,12 @@
       <c r="H14" s="7"/>
       <c r="I14" s="9"/>
       <c r="J14" s="11"/>
-      <c r="K14" s="13"/>
+      <c r="K14" s="7"/>
       <c r="L14" s="13"/>
       <c r="M14" s="13"/>
       <c r="N14" s="13"/>
       <c r="O14" s="13"/>
+      <c r="P14" s="13"/>
     </row>
     <row r="15" ht="84" customHeight="1">
       <c r="A15" s="6">
@@ -653,11 +718,12 @@
       <c r="H15" s="8"/>
       <c r="I15" s="10"/>
       <c r="J15" s="12"/>
-      <c r="K15" s="14"/>
+      <c r="K15" s="8"/>
       <c r="L15" s="14"/>
       <c r="M15" s="14"/>
       <c r="N15" s="14"/>
       <c r="O15" s="14"/>
+      <c r="P15" s="14"/>
     </row>
     <row r="16" ht="84" customHeight="1">
       <c r="A16" s="5">
@@ -672,11 +738,12 @@
       <c r="H16" s="7"/>
       <c r="I16" s="9"/>
       <c r="J16" s="11"/>
-      <c r="K16" s="13"/>
+      <c r="K16" s="7"/>
       <c r="L16" s="13"/>
       <c r="M16" s="13"/>
       <c r="N16" s="13"/>
       <c r="O16" s="13"/>
+      <c r="P16" s="13"/>
     </row>
     <row r="17" ht="84" customHeight="1">
       <c r="A17" s="6">
@@ -691,11 +758,12 @@
       <c r="H17" s="8"/>
       <c r="I17" s="10"/>
       <c r="J17" s="12"/>
-      <c r="K17" s="14"/>
+      <c r="K17" s="8"/>
       <c r="L17" s="14"/>
       <c r="M17" s="14"/>
       <c r="N17" s="14"/>
       <c r="O17" s="14"/>
+      <c r="P17" s="14"/>
     </row>
     <row r="18" ht="84" customHeight="1">
       <c r="A18" s="5">
@@ -710,11 +778,12 @@
       <c r="H18" s="7"/>
       <c r="I18" s="9"/>
       <c r="J18" s="11"/>
-      <c r="K18" s="13"/>
+      <c r="K18" s="7"/>
       <c r="L18" s="13"/>
       <c r="M18" s="13"/>
       <c r="N18" s="13"/>
       <c r="O18" s="13"/>
+      <c r="P18" s="13"/>
     </row>
     <row r="19" ht="84" customHeight="1">
       <c r="A19" s="6">
@@ -729,11 +798,12 @@
       <c r="H19" s="8"/>
       <c r="I19" s="10"/>
       <c r="J19" s="12"/>
-      <c r="K19" s="14"/>
+      <c r="K19" s="8"/>
       <c r="L19" s="14"/>
       <c r="M19" s="14"/>
       <c r="N19" s="14"/>
       <c r="O19" s="14"/>
+      <c r="P19" s="14"/>
     </row>
     <row r="20" ht="84" customHeight="1">
       <c r="A20" s="5">
@@ -748,11 +818,12 @@
       <c r="H20" s="7"/>
       <c r="I20" s="9"/>
       <c r="J20" s="11"/>
-      <c r="K20" s="13"/>
+      <c r="K20" s="7"/>
       <c r="L20" s="13"/>
       <c r="M20" s="13"/>
       <c r="N20" s="13"/>
       <c r="O20" s="13"/>
+      <c r="P20" s="13"/>
     </row>
     <row r="21" ht="84" customHeight="1">
       <c r="A21" s="6">
@@ -767,11 +838,12 @@
       <c r="H21" s="8"/>
       <c r="I21" s="10"/>
       <c r="J21" s="12"/>
-      <c r="K21" s="14"/>
+      <c r="K21" s="8"/>
       <c r="L21" s="14"/>
       <c r="M21" s="14"/>
       <c r="N21" s="14"/>
       <c r="O21" s="14"/>
+      <c r="P21" s="14"/>
     </row>
     <row r="22" ht="84" customHeight="1">
       <c r="A22" s="5">
@@ -786,11 +858,12 @@
       <c r="H22" s="7"/>
       <c r="I22" s="9"/>
       <c r="J22" s="11"/>
-      <c r="K22" s="13"/>
+      <c r="K22" s="7"/>
       <c r="L22" s="13"/>
       <c r="M22" s="13"/>
       <c r="N22" s="13"/>
       <c r="O22" s="13"/>
+      <c r="P22" s="13"/>
     </row>
     <row r="23" ht="84" customHeight="1">
       <c r="A23" s="6">
@@ -805,11 +878,12 @@
       <c r="H23" s="8"/>
       <c r="I23" s="10"/>
       <c r="J23" s="12"/>
-      <c r="K23" s="14"/>
+      <c r="K23" s="8"/>
       <c r="L23" s="14"/>
       <c r="M23" s="14"/>
       <c r="N23" s="14"/>
       <c r="O23" s="14"/>
+      <c r="P23" s="14"/>
     </row>
     <row r="24" ht="84" customHeight="1">
       <c r="A24" s="5">
@@ -824,11 +898,12 @@
       <c r="H24" s="7"/>
       <c r="I24" s="9"/>
       <c r="J24" s="11"/>
-      <c r="K24" s="13"/>
+      <c r="K24" s="7"/>
       <c r="L24" s="13"/>
       <c r="M24" s="13"/>
       <c r="N24" s="13"/>
       <c r="O24" s="13"/>
+      <c r="P24" s="13"/>
     </row>
     <row r="25" ht="84" customHeight="1">
       <c r="A25" s="6">
@@ -843,11 +918,12 @@
       <c r="H25" s="8"/>
       <c r="I25" s="10"/>
       <c r="J25" s="12"/>
-      <c r="K25" s="14"/>
+      <c r="K25" s="8"/>
       <c r="L25" s="14"/>
       <c r="M25" s="14"/>
       <c r="N25" s="14"/>
       <c r="O25" s="14"/>
+      <c r="P25" s="14"/>
     </row>
     <row r="26" ht="84" customHeight="1">
       <c r="A26" s="5">
@@ -862,11 +938,12 @@
       <c r="H26" s="7"/>
       <c r="I26" s="9"/>
       <c r="J26" s="11"/>
-      <c r="K26" s="13"/>
+      <c r="K26" s="7"/>
       <c r="L26" s="13"/>
       <c r="M26" s="13"/>
       <c r="N26" s="13"/>
       <c r="O26" s="13"/>
+      <c r="P26" s="13"/>
     </row>
     <row r="27" ht="84" customHeight="1">
       <c r="A27" s="6">
@@ -881,11 +958,12 @@
       <c r="H27" s="8"/>
       <c r="I27" s="10"/>
       <c r="J27" s="12"/>
-      <c r="K27" s="14"/>
+      <c r="K27" s="8"/>
       <c r="L27" s="14"/>
       <c r="M27" s="14"/>
       <c r="N27" s="14"/>
       <c r="O27" s="14"/>
+      <c r="P27" s="14"/>
     </row>
     <row r="28" ht="84" customHeight="1">
       <c r="A28" s="5">
@@ -900,11 +978,12 @@
       <c r="H28" s="7"/>
       <c r="I28" s="9"/>
       <c r="J28" s="11"/>
-      <c r="K28" s="13"/>
+      <c r="K28" s="7"/>
       <c r="L28" s="13"/>
       <c r="M28" s="13"/>
       <c r="N28" s="13"/>
       <c r="O28" s="13"/>
+      <c r="P28" s="13"/>
     </row>
     <row r="29" ht="84" customHeight="1">
       <c r="A29" s="6">
@@ -919,11 +998,12 @@
       <c r="H29" s="8"/>
       <c r="I29" s="10"/>
       <c r="J29" s="12"/>
-      <c r="K29" s="14"/>
+      <c r="K29" s="8"/>
       <c r="L29" s="14"/>
       <c r="M29" s="14"/>
       <c r="N29" s="14"/>
       <c r="O29" s="14"/>
+      <c r="P29" s="14"/>
     </row>
     <row r="30" ht="84" customHeight="1">
       <c r="A30" s="5">
@@ -938,11 +1018,12 @@
       <c r="H30" s="7"/>
       <c r="I30" s="9"/>
       <c r="J30" s="11"/>
-      <c r="K30" s="13"/>
+      <c r="K30" s="7"/>
       <c r="L30" s="13"/>
       <c r="M30" s="13"/>
       <c r="N30" s="13"/>
       <c r="O30" s="13"/>
+      <c r="P30" s="13"/>
     </row>
     <row r="31" ht="84" customHeight="1">
       <c r="A31" s="6">
@@ -957,11 +1038,12 @@
       <c r="H31" s="8"/>
       <c r="I31" s="10"/>
       <c r="J31" s="12"/>
-      <c r="K31" s="14"/>
+      <c r="K31" s="8"/>
       <c r="L31" s="14"/>
       <c r="M31" s="14"/>
       <c r="N31" s="14"/>
       <c r="O31" s="14"/>
+      <c r="P31" s="14"/>
     </row>
     <row r="32" ht="84" customHeight="1">
       <c r="A32" s="5">
@@ -976,11 +1058,12 @@
       <c r="H32" s="7"/>
       <c r="I32" s="9"/>
       <c r="J32" s="11"/>
-      <c r="K32" s="13"/>
+      <c r="K32" s="7"/>
       <c r="L32" s="13"/>
       <c r="M32" s="13"/>
       <c r="N32" s="13"/>
       <c r="O32" s="13"/>
+      <c r="P32" s="13"/>
     </row>
     <row r="33" ht="84" customHeight="1">
       <c r="A33" s="6">
@@ -995,18 +1078,38 @@
       <c r="H33" s="8"/>
       <c r="I33" s="10"/>
       <c r="J33" s="12"/>
-      <c r="K33" s="14"/>
+      <c r="K33" s="8"/>
       <c r="L33" s="14"/>
       <c r="M33" s="14"/>
       <c r="N33" s="14"/>
       <c r="O33" s="14"/>
+      <c r="P33" s="14"/>
     </row>
   </sheetData>
-  <autoFilter ref="A3:O33"/>
+  <autoFilter ref="A3:P33"/>
   <mergeCells count="2">
-    <mergeCell ref="A1:O1"/>
-    <mergeCell ref="A2:O2"/>
+    <mergeCell ref="A1:P1"/>
+    <mergeCell ref="A2:P2"/>
   </mergeCells>
+  <conditionalFormatting sqref="K4:K33">
+    <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
+      <formula>"New"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
+      <formula>"In process"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="2" priority="3" operator="equal">
+      <formula>"Done"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="3" priority="4" operator="equal">
+      <formula>"Cancelled"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="warning" errorTitle="Status" error="Use New, In process, Done or Cancelled." sqref="K4:K33">
+      <formula1>"New,In process,Done,Cancelled"</formula1>
+    </dataValidation>
+  </dataValidations>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.5" header="0.2" footer="0.25"/>
   <pageSetup paperSize="9" orientation="landscape" fitToWidth="1" fitToHeight="0"/>
@@ -1014,7 +1117,7 @@
     <oddFooter>&amp;C&amp;"Calibri,Regular"&amp;9ACP4U  -  &amp;P / &amp;N</oddFooter>
   </headerFooter>
   <ignoredErrors>
-    <ignoredError sqref="A4:O33" numberStoredAsText="1"/>
+    <ignoredError sqref="A4:P33" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>